<commit_message>
Fix missing pull up resistors on stemma qt port
</commit_message>
<xml_diff>
--- a/pcb/production/pickandplace_jlcpcb.xlsx
+++ b/pcb/production/pickandplace_jlcpcb.xlsx
@@ -4,14 +4,14 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="PickAndPlace_PCB1_2026-08-18" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="PickAndPlace_PCB1_2026-08-26" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1130" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1154" uniqueCount="422">
   <si>
     <t>Designator</t>
   </si>
@@ -1259,6 +1259,24 @@
   </si>
   <si>
     <t>DNP</t>
+  </si>
+  <si>
+    <t>R56</t>
+  </si>
+  <si>
+    <t>4.699mm</t>
+  </si>
+  <si>
+    <t>19.304mm</t>
+  </si>
+  <si>
+    <t>19.737mm</t>
+  </si>
+  <si>
+    <t>R57</t>
+  </si>
+  <si>
+    <t>3.302mm</t>
   </si>
 </sst>
 </file>
@@ -1635,7 +1653,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N94"/>
+  <dimension ref="A1:N96"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="14" width="20" customWidth="1"/>
@@ -5777,6 +5795,94 @@
         <v>415</v>
       </c>
     </row>
+    <row r="95" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>416</v>
+      </c>
+      <c r="B95" t="s">
+        <v>169</v>
+      </c>
+      <c r="C95" t="s">
+        <v>170</v>
+      </c>
+      <c r="D95" t="s">
+        <v>417</v>
+      </c>
+      <c r="E95" t="s">
+        <v>418</v>
+      </c>
+      <c r="F95" t="s">
+        <v>417</v>
+      </c>
+      <c r="G95" t="s">
+        <v>418</v>
+      </c>
+      <c r="H95" t="s">
+        <v>417</v>
+      </c>
+      <c r="I95" t="s">
+        <v>419</v>
+      </c>
+      <c r="J95">
+        <v>2</v>
+      </c>
+      <c r="K95" t="s">
+        <v>20</v>
+      </c>
+      <c r="L95">
+        <v>270</v>
+      </c>
+      <c r="M95" t="s">
+        <v>21</v>
+      </c>
+      <c r="N95" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="96" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>420</v>
+      </c>
+      <c r="B96" t="s">
+        <v>169</v>
+      </c>
+      <c r="C96" t="s">
+        <v>170</v>
+      </c>
+      <c r="D96" t="s">
+        <v>421</v>
+      </c>
+      <c r="E96" t="s">
+        <v>418</v>
+      </c>
+      <c r="F96" t="s">
+        <v>421</v>
+      </c>
+      <c r="G96" t="s">
+        <v>418</v>
+      </c>
+      <c r="H96" t="s">
+        <v>421</v>
+      </c>
+      <c r="I96" t="s">
+        <v>419</v>
+      </c>
+      <c r="J96">
+        <v>2</v>
+      </c>
+      <c r="K96" t="s">
+        <v>20</v>
+      </c>
+      <c r="L96">
+        <v>270</v>
+      </c>
+      <c r="M96" t="s">
+        <v>21</v>
+      </c>
+      <c r="N96" t="s">
+        <v>174</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>